<commit_message>
LSOA to Ward lookup
</commit_message>
<xml_diff>
--- a/resources/sheffield_transport_datasets.xlsx
+++ b/resources/sheffield_transport_datasets.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lp41455\repo\transport-env-typology\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lp41455\repo\transport-env-typology\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{469F4C4F-A9DD-458D-B43F-2689A3F80382}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7770C059-63EC-42B6-88B7-0393E0D3221E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57480" yWindow="-1095" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw datasets" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="111">
   <si>
     <t>Raw datasets used by the pipeline</t>
   </si>
@@ -362,6 +362,18 @@
   </si>
   <si>
     <t>Indices of Deprivation (2025)</t>
+  </si>
+  <si>
+    <t>LSOA (2021) to Electoral Ward (2025) Best Fit Lookup for Sheffield</t>
+  </si>
+  <si>
+    <t>ONS Open Geography Portal API: https://geoportal.statistics.gov.uk/datasets/ons::lsoa-2021-to-electoral-ward-2025-to-lad-2025-best-fit-lookup-in-ew-v2/about</t>
+  </si>
+  <si>
+    <t>df_lsoa_ward</t>
+  </si>
+  <si>
+    <t>Sheffield LSOA to Ward lookup</t>
   </si>
 </sst>
 </file>
@@ -554,8 +566,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="RawDatasetsTable" displayName="RawDatasetsTable" ref="A4:E20">
-  <autoFilter ref="A4:E20" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="RawDatasetsTable" displayName="RawDatasetsTable" ref="A4:E21">
+  <autoFilter ref="A4:E21" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Dataset name"/>
     <tableColumn id="4" xr3:uid="{1EB550B7-E986-4A9C-A7D1-F4CFC42610FC}" name="Data frame" dataDxfId="1"/>
@@ -867,7 +879,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="35.81640625" customWidth="1"/>
@@ -948,33 +960,33 @@
     </row>
     <row r="7" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
-        <v>5</v>
+        <v>110</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>66</v>
+        <v>109</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>6</v>
+        <v>107</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>86</v>
+        <v>108</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E8" s="8" t="s">
         <v>86</v>
@@ -982,16 +994,16 @@
     </row>
     <row r="9" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E9" s="7" t="s">
         <v>86</v>
@@ -999,16 +1011,16 @@
     </row>
     <row r="10" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E10" s="8" t="s">
         <v>86</v>
@@ -1016,16 +1028,16 @@
     </row>
     <row r="11" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>88</v>
+        <v>12</v>
       </c>
       <c r="E11" s="7" t="s">
         <v>86</v>
@@ -1033,135 +1045,135 @@
     </row>
     <row r="12" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>58</v>
+        <v>73</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>98</v>
+        <v>74</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C13" s="9" t="s">
         <v>98</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>16</v>
+        <v>89</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C14" s="10" t="s">
         <v>98</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>19</v>
+        <v>85</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="9" t="s">
-        <v>106</v>
+        <v>17</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>102</v>
+        <v>60</v>
       </c>
       <c r="C15" s="9" t="s">
         <v>98</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>100</v>
+        <v>18</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>101</v>
+        <v>19</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
-        <v>20</v>
+        <v>106</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>75</v>
+        <v>102</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>76</v>
+        <v>98</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>21</v>
+        <v>100</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>22</v>
+        <v>101</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="4" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>92</v>
+        <v>25</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>90</v>
+        <v>27</v>
       </c>
       <c r="E19" s="7" t="s">
         <v>92</v>
@@ -1169,18 +1181,35 @@
     </row>
     <row r="20" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="D20" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="E20" s="8" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B21" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="C21" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="D20" s="10" t="s">
+      <c r="D21" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="E20" s="8" t="s">
+      <c r="E21" s="7" t="s">
         <v>92</v>
       </c>
     </row>

</xml_diff>